<commit_message>
radar: coleta de 2026-09-07
</commit_message>
<xml_diff>
--- a/dados/licitacoes.xlsx
+++ b/dados/licitacoes.xlsx
@@ -21,7 +21,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'radar'!$A$1:$M$38</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'metricas'!$A$1:$R$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'municipios'!$A$1:$G$39</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'falhas_coleta'!$A$1:$G$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'falhas_coleta'!$A$1:$G$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -35492,12 +35492,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>46377800000127-1-003319/2026</t>
+          <t>65712002000159-1-000023/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Fernandópolis</t>
+          <t>Aspásia</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -35505,7 +35505,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>14</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -35518,20 +35518,20 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prestação de serviço de manutenção corretiva e preventiva em ar condicionado </t>
+          <t>Registro de Preços para contratação de empresa especializada para o fornecimento parcelado de pneus e bicos novos e prestação de serviços de desmontagem e montagem, alinhamento e balanceamento, destinados à manutenção da frota de veículos e máquinas do município de Aspásia-SP.</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>122500</v>
+        <v>665093.99</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-08-19T08:00:00</t>
+          <t>2026-08-20T08:00:00</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-09-03T09:00:00</t>
+          <t>2026-09-08T08:00:00</t>
         </is>
       </c>
       <c r="K2" t="n">
@@ -35539,19 +35539,19 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/compras/acompanhamento-compra?compra=18014705000462026</t>
+          <t>https://bllcompras.com/Process/ProcessView?param1=[gkz]i44RbKG8E9oJqSdtI6Sh4VkzESZ_8CfAACb4t7PThlEYD45sizcqDmpqW0HHsaZIDhYFYz0NE509__WgUwQg0krDq0X5mU0MdVNA8amx4aI=</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>SAO PAULO SECRETARIA DA SEGURANCA PUBLICA</t>
+          <t>MUNICIPIO DE ASPASIA</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>47842836000105-1-000151/2026</t>
+          <t>47842836000105-1-000155/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -35564,7 +35564,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>41</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -35577,20 +35577,20 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA O FORNECIMENTO DE KITS DE LANCHES, BEBIDAS E INSUMOS, INCLUINDO O TRANSPORTE E ENTREGA EM TODOS OS PONTOS ESPECIFICADOS NO TERMO DE REFERÊNCIA, BEM COMO PARA A PRESTAÇÃO DE SERVIÇOS DE REFEIÇÃO PRONTA EM RESTAURANTE NA MODALIDADE SELF-SERVICE, VISANDO AO ATENDIMENTO DAS NECESSIDADES LOGÍSTICAS E OPERACIONAIS DO JUÍZO ELEITORAL DA 150ª ZONA ELEITORAL NO TREINAMENTO DE MESÁRIOS E NO APOIO ÀS ELEIÇÕES GERAIS DE 2026 (1º E 2º TURNOS) NO MUNICÍPIO DE FERNANDÓPOLIS/SP</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA PRESTAÇÃO CONTÍNUA DE SOLUÇÃO INTEGRADA DE RADIOCOMUNICAÇÃO DIGITAL POC, INCLUINDO LOCAÇÃO DE EQUIPAMENTOS, SOFTWARE DE GRAVAÇÃO E GESTÃO OPERACIONAL, CONECTIVIDADE, SUPORTE TÉCNICO E MANUTENÇÃO, PARA ATENDIMENTO DO SAMU 192 REGIONAL FERNANDÓPOLIS</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>129102.12</v>
+        <v>61816.08</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-08-17T08:00:00</t>
+          <t>2026-08-19T08:00:00</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-09-03T08:29:00</t>
+          <t>2026-09-08T08:29:00</t>
         </is>
       </c>
       <c r="K3" t="n">
@@ -35598,7 +35598,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/compras/acompanhamento-compra?compra=98641105000382026</t>
+          <t>https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/compras/acompanhamento-compra?compra=98641105000412026</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -35610,12 +35610,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>45116092000108-1-000109/2026</t>
+          <t>46377800000127-1-003566/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Meridiano</t>
+          <t>Fernandópolis</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -35623,33 +35623,33 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>48</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Pregão - Presencial</t>
+          <t>Pregão - Eletrônico</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA A PRESTAÇÃO DE SERVIÇOS MÉDICOS NA ESPECIALIDADE DE GINECOLOGIA E OBSTETRÍCIA, MEDIANTE DISPONIBILIZAÇÃO DE PROFISSIONAL MÉDICO DEVIDAMENTE HABILITADO, PARA REALIZAÇÃO DE CONSULTAS, ATENDIMENTOS, AVALIAÇÕES, ACOMPANHAMENTO CLÍNICO E DEMAIS PROCEDIMENTOS COMPATÍVEIS COM A ESPECIALIDADE, DESTINADOS ÀS USUÁRIAS DA REDE MUNICIPAL DE SAÚDE DE MERIDIANO/SP</t>
+          <t>AQUISIÇÃO DE MATERIAL PERMANENTE</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>106488</v>
+        <v>26498.46</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-09-03T00:01:00</t>
+          <t>2026-08-25T08:00:00</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-09-03T23:59:00</t>
+          <t>2026-09-08T09:00:00</t>
         </is>
       </c>
       <c r="K4" t="n">
@@ -35657,24 +35657,24 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>https://meridiano.sp.gov.br/licitacao/</t>
+          <t>https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/compras/acompanhamento-compra?compra=18014705000482026</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE MERIDIANO</t>
+          <t>SAO PAULO SECRETARIA DA SEGURANCA PUBLICA</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>45116712000109-1-000049/2026</t>
+          <t>45138088000140-1-000005/2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>São João das Duas Pontes</t>
+          <t>Santana da Ponte Pensa</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -35682,7 +35682,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>014</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -35695,48 +35695,53 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>ELABORAÇÃO DE ATA DE REGISTRO DE PREÇOS PARA FUTURA E EVENTUAL AQUISIÇÃO DE GÊNEROS ALIMENTÍCIOS, DESTINADOS À ALIMENTAÇÃO ESCOLAR DAS ESCOLAS MUNICIPAIS E ESTADUAL, BEM COMO AO ATENDIMENTO DAS NECESSIDADES DAS DIVERSAS DIRETORIAS DO MUNICÍPIO QUE DEMANDEM O FORNECIMENTO DE GÊNEROS ALIMENTÍCIOS, PELO PERÍODO DE 12 (DOZE) MESES.</t>
+          <t>AQUISIÇÃO DE (01) UM VEÍCULO PICK-UP, ZERO KM, PRIMEIRO EMPLACAMENTO, PARA ATENDER AS NECESSIDADES DA SECRETARIA MUNICIPAL DE SAÚDE DO MUNICÍPIO DE SANTANA DA PONTE PENSA.</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>255533.14</v>
+        <v>229902.55</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-08-24T08:00:00</t>
+          <t>2026-08-26T08:00:00</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-03T08:59:00</t>
+          <t>2026-09-08T08:00:00</t>
         </is>
       </c>
       <c r="K5" t="n">
         <v>0</v>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>https://bllcompras.com/Process/ProcessView?param1=[gkz]Zc0JylBKo1JG2gT7EY9UZRj8hNFcLCGxTa88/fZstJSEJqAofOH7MjcCSf4ZZRWkbiEHAOFuJ5DOro/AMSClwfAD12P5RAVpzImGJl/PM6k=</t>
+        </is>
+      </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE SAO JOAO DAS DUAS PONTES</t>
+          <t>MUNICIPIO DE SANTANA DA PONTE PENSA</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>45138070000149-1-000780/2026</t>
+          <t>45139482000101-1-000013/2026</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Santa Fé do Sul</t>
+          <t>Turmalina</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>17</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -35749,20 +35754,20 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Registro de preços para aquisição de medicamentos para atendimento das demanda da farmacia municipal e demandas judiciais.</t>
+          <t>Ata de registro de preço para futura e eventual aquisição de utensílios de cozinha destinados ao atendimento das demandas das Escolas Municipais, Unidades de Saúde, Secretaria de Assistência Social e demais setores da Administração Municipal.</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>2531636.26</v>
+        <v>103402.98</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-08-24T09:00:00</t>
+          <t>2026-08-11T15:00:00</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-04T08:00:00</t>
+          <t>2026-09-08T08:00:00</t>
         </is>
       </c>
       <c r="K6" t="n">
@@ -35770,24 +35775,24 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/compras/acompanhamento-compra?compra=98703305000772026</t>
+          <t>https://bllcompras.com/Process/ProcessView?param1=[gkz]N0wBsRugqEYND870UfbnyD0/_ysDfol_QeTbKmEoo4AHv33QRORAgb4lL/L7V7adIloPW1LwTLPlvbBu//DxKxic2se6ey_Ga28uyEu_ltY=</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE SANTA FE DO SUL</t>
+          <t>MUNICIPIO DE TURMALINA</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>65712002000159-1-000024/2026</t>
+          <t>45116290000171-1-000071/2026</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Aspásia</t>
+          <t>Mira Estrela</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -35795,7 +35800,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>26</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -35808,45 +35813,40 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Contratação de empresa para fornecimento de 01 (um) veículo automotor de passeio 0 km, 03 (três) lixeiras e 01 (um) tablet, destinados ao atendimento das necessidades do Departamento de Saúde do município de Aspásia/SP, conforme proposta nº 13870352000126001/2026, firmada entre o Ministério da Saúde e o município de Aspásia/SP.</t>
+          <t>SOLICITÇÃO DE PREGÃO DE MEDICAMENTOS CONTROLADO, GERAL E INJETAVEIS</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>122348.38</v>
+        <v>4998762.9</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-08-24T08:00:00</t>
+          <t>2026-08-25T08:00:00</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-04T08:00:00</t>
+          <t>2026-09-09T08:30:00</t>
         </is>
       </c>
       <c r="K7" t="n">
         <v>0</v>
       </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>https://bllcompras.com/Process/ProcessView?param1=[gkz]4jJu5RffCYlYdps5LYfbR0JHx0oo9ahOA4uYtfW3spcbkFtm8dXlcESvWAickcC71IQWJEcN_vAtjWaGD8OwbilZw9ku4N5Bkf4NOm21WaU=</t>
-        </is>
-      </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE ASPASIA</t>
+          <t>MUNICIPIO DE MIRA ESTRELA</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>47842836000105-1-000152/2026</t>
+          <t>46609731000130-1-000009/2026</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Fernandópolis</t>
+          <t>Palmeira d'Oeste</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -35854,7 +35854,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>0011/26</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -35867,20 +35867,20 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>ELABORAÇÃO DE ATA DE REGISTRO DE PREÇOS PARA CONTRATAÇÃO DE EMPRESA ESPECIALIZADA EM SERVIÇOS TÉCNICOS DE OPERAÇÃO DE SOM E ILUMINAÇÃO, COM PREVISÃO DE CONSUMO PARCELADAMENTE NO DECORRER DE 12 (DOZE) MESES</t>
+          <t>AQUISIÇÃO DE MATERIAL PERMANENTE E EQUIPAMENTOS PARA ATENDER AS DEMANDAS DAS EMENDAS IMPOSITIVAS DO MUNICÍPIO DE PALMEIRA D’ OESTE</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>231251.25</v>
+        <v>213739.13</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-08-17T08:00:00</t>
+          <t>2026-08-25T08:00:00</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-04T08:29:00</t>
+          <t>2026-09-09T07:55:00</t>
         </is>
       </c>
       <c r="K8" t="n">
@@ -35888,24 +35888,24 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/compras/acompanhamento-compra?compra=98641105000392026</t>
+          <t>https://bllcompras.com/Process/ProcessView?param1=[gkz]QnI_GPPDwUvDgOdOlJLDJhZZiulGuLBl9ABAquFHbN8NuY8msOBhFE2geRC3Qh4U8jymTBYarlI4L6jhmqtI6kPr7M6M3vExjtzomNkyN2k=</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE FERNANDOPOLIS</t>
+          <t>MUNICIPIO DE PALMEIRA D'OESTE</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>01611211000123-1-000048/2026</t>
+          <t>45135043000112-1-000044/2026</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Santa Salete</t>
+          <t>Rubinéia</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -35913,33 +35913,33 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>16</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Pregão - Eletrônico</t>
+          <t>Pregão - Presencial</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE LABORATÓRIO DE ANÁLISES CLÍNICAS PARA REALIZAÇÃO DE COLETA E ANALISES DE EXAMES LABORATORIAIS</t>
+          <t>SERVIÇOS DE MANUTENÇÃO E INSTALAÇÃO DE SISTEMAS DE AR-CONDICIONADO E CLIMATIZADORES, COM REPOSIÇÃO DE PEÇAS</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>222037.4</v>
+        <v>354029.86</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-08-20T08:30:00</t>
+          <t>2026-08-20T15:00:00</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-04T08:30:00</t>
+          <t>2026-09-10T09:15:00</t>
         </is>
       </c>
       <c r="K9" t="n">
@@ -35947,19 +35947,19 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE SANTA SALETE</t>
+          <t>MUNICIPIO DE RUBINEIA</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>65712002000159-1-000023/2026</t>
+          <t>45135530000185-1-000043/2026</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Aspásia</t>
+          <t>Santa Albertina</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -35967,7 +35967,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -35980,45 +35980,40 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Registro de Preços para contratação de empresa especializada para o fornecimento parcelado de pneus e bicos novos e prestação de serviços de desmontagem e montagem, alinhamento e balanceamento, destinados à manutenção da frota de veículos e máquinas do município de Aspásia-SP.</t>
+          <t>SOLICITAÇÃO GERADA PARA COTAÇÃO DE VÁRIAS SOLICITAÇÕES</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>665093.99</v>
+        <v>1217853.48</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-08-20T08:00:00</t>
+          <t>2026-08-26T08:00:00</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-08T08:00:00</t>
+          <t>2026-09-10T08:30:00</t>
         </is>
       </c>
       <c r="K10" t="n">
         <v>0</v>
       </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>https://bllcompras.com/Process/ProcessView?param1=[gkz]i44RbKG8E9oJqSdtI6Sh4VkzESZ_8CfAACb4t7PThlEYD45sizcqDmpqW0HHsaZIDhYFYz0NE509__WgUwQg0krDq0X5mU0MdVNA8amx4aI=</t>
-        </is>
-      </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE ASPASIA</t>
+          <t>MUNICIPIO DE SANTA ALBERTINA</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>47842836000105-1-000155/2026</t>
+          <t>65712002000159-1-000027/2026</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Fernandópolis</t>
+          <t>Aspásia</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -36026,12 +36021,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>02</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Pregão - Eletrônico</t>
+          <t>Dispensa</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -36039,20 +36034,20 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA PRESTAÇÃO CONTÍNUA DE SOLUÇÃO INTEGRADA DE RADIOCOMUNICAÇÃO DIGITAL POC, INCLUINDO LOCAÇÃO DE EQUIPAMENTOS, SOFTWARE DE GRAVAÇÃO E GESTÃO OPERACIONAL, CONECTIVIDADE, SUPORTE TÉCNICO E MANUTENÇÃO, PARA ATENDIMENTO DO SAMU 192 REGIONAL FERNANDÓPOLIS</t>
+          <t xml:space="preserve">Contratação de empresa especializada para o fornecimento de violões, ukuleles e capas para ukuleles, destinados às atividades da oficina de música promovida pelo Município de Aspásia/SP, visando assegurar condições adequadas para a realização das aulas, o desenvolvimento das habilidades musicais dos alunos e o fortalecimento das ações de formação e promoção cultural desenvolvidas pela Administração Municipal.  </t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>61816.08</v>
+        <v>9779.610000000001</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-08-19T08:00:00</t>
+          <t>2026-09-04T08:00:00</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-08T08:29:00</t>
+          <t>2026-09-10T08:00:00</t>
         </is>
       </c>
       <c r="K11" t="n">
@@ -36060,24 +36055,24 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/compras/acompanhamento-compra?compra=98641105000412026</t>
+          <t>https://bllcompras.com/Process/ProcessView?param1=[gkz]7Wibt1ZEawQQa4ymZcalR_ZEne7pDiHyVK57rz16w49ss5QlfD9DUCIo6o1gQCowk6VBXwjwYmWyxM2Bdf8me4M4cPKPwQV2MJg8TdTbbv4=</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE FERNANDOPOLIS</t>
+          <t>MUNICIPIO DE ASPASIA</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>46377800000127-1-003566/2026</t>
+          <t>51842177000176-1-000009/2026</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Fernandópolis</t>
+          <t>Populina</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -36085,7 +36080,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -36098,20 +36093,20 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>AQUISIÇÃO DE MATERIAL PERMANENTE</t>
+          <t>Registro de preços para futura e eventual aquisição, com instalação, de playgrounds, brinquedos infantis, equipamentos recreativos e mobiliário de apoio, destinados a praças, parques, escolas e demais espaços públicos municipais de Populina/SP.</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>26498.46</v>
+        <v>2237327.4</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-08-25T08:00:00</t>
+          <t>2026-08-26T08:00:00</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-08T09:00:00</t>
+          <t>2026-09-11T08:25:00</t>
         </is>
       </c>
       <c r="K12" t="n">
@@ -36119,24 +36114,24 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/compras/acompanhamento-compra?compra=18014705000482026</t>
+          <t>https://bllcompras.com/Process/ProcessView?param1=[gkz]bLezG7PRY7kJ7HUtk7XrKi8hDh5fHQ8eun9/MHtyLQ04gxN3BLr9J8rvwQ/KeKtJFkMnFHKfUVMoJVWokccurrPTtpguXan7eH8UyRlHbHw=</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>SAO PAULO SECRETARIA DA SEGURANCA PUBLICA</t>
+          <t>MUNICIPIO DE POPULINA</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>45138088000140-1-000005/2026</t>
+          <t>01611210000189-1-000039/2026</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Santana da Ponte Pensa</t>
+          <t>Vitória Brasil</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -36144,7 +36139,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>014</t>
+          <t>019</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -36157,20 +36152,20 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>AQUISIÇÃO DE (01) UM VEÍCULO PICK-UP, ZERO KM, PRIMEIRO EMPLACAMENTO, PARA ATENDER AS NECESSIDADES DA SECRETARIA MUNICIPAL DE SAÚDE DO MUNICÍPIO DE SANTANA DA PONTE PENSA.</t>
+          <t>Contratação de empresa especializada para prestação continuada de serviços técnicos profissionais de engenharia civil, mediante disponibilização de profissional legalmente habilitado e registrado no CREA, para atendimento das demandas técnicas do Município de Vitória Brasil/SP, conforme especificações e condições estabelecidas no Termo de Referência.</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>229902.55</v>
+        <v>72000</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-08-26T08:00:00</t>
+          <t>2026-08-26T07:00:00</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-08T08:00:00</t>
+          <t>2026-09-11T07:00:00</t>
         </is>
       </c>
       <c r="K13" t="n">
@@ -36178,32 +36173,32 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>https://bllcompras.com/Process/ProcessView?param1=[gkz]Zc0JylBKo1JG2gT7EY9UZRj8hNFcLCGxTa88/fZstJSEJqAofOH7MjcCSf4ZZRWkbiEHAOFuJ5DOro/AMSClwfAD12P5RAVpzImGJl/PM6k=</t>
+          <t>https://bllcompras.com/Process/ProcessView?param1=[gkz]vQQuhlx2Pl8lkR4jblHBp53gsyiYaUO5R79qyHqzmfBAXAgoaWDIYQNetaVTV6wokPn_VoeOaP31PgAi8W9JkZoK42fYxR_Q3rLDM3pZlz4=</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE SANTANA DA PONTE PENSA</t>
+          <t>MUNICIPIO DE VITORIA BRASIL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>45139482000101-1-000013/2026</t>
+          <t>45138070000149-1-000794/2026</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Turmalina</t>
+          <t>Santa Fé do Sul</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -36216,20 +36211,20 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Ata de registro de preço para futura e eventual aquisição de utensílios de cozinha destinados ao atendimento das demandas das Escolas Municipais, Unidades de Saúde, Secretaria de Assistência Social e demais setores da Administração Municipal.</t>
+          <t>Aquisição de material permanente do tipo arma de fogo, destinados ao aparelhamento da Guarda Civil Municipal</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>103402.98</v>
+        <v>214982.55</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-08-11T15:00:00</t>
+          <t>2026-09-01T08:00:00</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-08T08:00:00</t>
+          <t>2026-09-14T08:00:00</t>
         </is>
       </c>
       <c r="K14" t="n">
@@ -36237,24 +36232,24 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>https://bllcompras.com/Process/ProcessView?param1=[gkz]N0wBsRugqEYND870UfbnyD0/_ysDfol_QeTbKmEoo4AHv33QRORAgb4lL/L7V7adIloPW1LwTLPlvbBu//DxKxic2se6ey_Ga28uyEu_ltY=</t>
+          <t>https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/compras/acompanhamento-compra?compra=98703305000012026</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE TURMALINA</t>
+          <t>MUNICIPIO DE SANTA FE DO SUL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>45116290000171-1-000071/2026</t>
+          <t>46609731000130-1-000010/2026</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Mira Estrela</t>
+          <t>Palmeira d'Oeste</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -36262,7 +36257,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>0012/26</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -36275,40 +36270,45 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>SOLICITÇÃO DE PREGÃO DE MEDICAMENTOS CONTROLADO, GERAL E INJETAVEIS</t>
+          <t>Registro de preço para futura e eventual aquisição e fornecimento de materiais hospitalares e injetáveis (ampolas) que serão utilizados nas Unidades Básicas de Saúde do município de Palmeira D’Oeste</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>4998762.9</v>
+        <v>1389925.25</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-08-25T08:00:00</t>
+          <t>2026-08-28T08:00:00</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-09T08:30:00</t>
+          <t>2026-09-15T07:55:00</t>
         </is>
       </c>
       <c r="K15" t="n">
         <v>0</v>
       </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>https://bllcompras.com/Process/ProcessView?param1=[gkz]l2ky7JpCrcgDbj_wLQNaUs/Mz/47PiTcEIcmcwf6lBs4uuoJI5JXsJ_Ups37yV8xnqw04gNabtq9EQoZRGeClFx0zNFKTnizlwfbEv/M2IM=</t>
+        </is>
+      </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE MIRA ESTRELA</t>
+          <t>MUNICIPIO DE PALMEIRA D'OESTE</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>46609731000130-1-000009/2026</t>
+          <t>46611117000102-1-000035/2026</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Palmeira d'Oeste</t>
+          <t>Urânia</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -36316,7 +36316,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0011/26</t>
+          <t>024</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -36329,20 +36329,20 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>AQUISIÇÃO DE MATERIAL PERMANENTE E EQUIPAMENTOS PARA ATENDER AS DEMANDAS DAS EMENDAS IMPOSITIVAS DO MUNICÍPIO DE PALMEIRA D’ OESTE</t>
+          <t>Contratação de empresa especializada para prestações de serviços mecânicos com fornecimento de peças para os seguintes veículos da frota municipal: FORD CAMINHÃO PIPA– Placa BFY2619 e ONIBUS VOLARE DW9 – Placa FQL1B98, pertencentes ao Município de Urânia/SP.</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>213739.13</v>
+        <v>35351.29</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-08-25T08:00:00</t>
+          <t>2026-09-01T09:00:00</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-09T07:55:00</t>
+          <t>2026-09-15T08:50:00</t>
         </is>
       </c>
       <c r="K16" t="n">
@@ -36350,24 +36350,24 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>https://bllcompras.com/Process/ProcessView?param1=[gkz]QnI_GPPDwUvDgOdOlJLDJhZZiulGuLBl9ABAquFHbN8NuY8msOBhFE2geRC3Qh4U8jymTBYarlI4L6jhmqtI6kPr7M6M3vExjtzomNkyN2k=</t>
+          <t>https://bllcompras.com/Process/ProcessView?param1=[gkz]jqtYlnxx02/zyCYX3kMbJ7UZt703DK0ewrudwGqCXRJlwWEUMxkpBqjwyPOSwmbnA_gUzilGP86b0FjDqmllHvDzbYRj6mOcMGzhbs8wzJM=</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE PALMEIRA D'OESTE</t>
+          <t>MUNICIPIO DE URANIA</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>45135043000112-1-000044/2026</t>
+          <t>45116712000109-1-000050/2026</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Rubinéia</t>
+          <t>São João das Duas Pontes</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -36375,33 +36375,33 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>23</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Pregão - Presencial</t>
+          <t>Pregão - Eletrônico</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>SERVIÇOS DE MANUTENÇÃO E INSTALAÇÃO DE SISTEMAS DE AR-CONDICIONADO E CLIMATIZADORES, COM REPOSIÇÃO DE PEÇAS</t>
+          <t>ELABORAÇÃO DE ATA DE REGISTRO DE PREÇOS PARA FUTURA E EVENTUAL AQUISIÇÃO PARCELADA DE MEDICAMENTOS, DESTINADOS AO ABASTECIMENTO DA FARMÁCIA MUNICIPAL E AO ATENDI-MENTO DOS PACIENTES USUÁRIOS DO SUS DO MUNICÍPIO DE SÃO JOÃO DAS DUAS PONTES/SP, PELO PERÍODO ESTIMADO DE 12 (DOZE) MESES’’.</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>354029.86</v>
+        <v>118801</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-08-20T15:00:00</t>
+          <t>2026-09-02T08:00:00</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-10T09:15:00</t>
+          <t>2026-09-15T08:59:00</t>
         </is>
       </c>
       <c r="K17" t="n">
@@ -36409,19 +36409,19 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE RUBINEIA</t>
+          <t>MUNICIPIO DE SAO JOAO DAS DUAS PONTES</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>45135530000185-1-000043/2026</t>
+          <t>45116712000109-1-000051/2026</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Santa Albertina</t>
+          <t>São João das Duas Pontes</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -36429,7 +36429,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>22</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -36442,20 +36442,20 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>SOLICITAÇÃO GERADA PARA COTAÇÃO DE VÁRIAS SOLICITAÇÕES</t>
+          <t>ELABORAÇÃO DE ATA DE REGISTRO DE PREÇOS PARA FUTURA E EVENTUAL AQUISIÇÃO DE EQUIPAMENTOS E DISPOSITIVOS TECNOLÓGICOS, INCLUINDO ITENS FRACASSADOS E NOVOS, PARA ATENDIMENTO DAS NECESSIDADES DOS DIVERSOS SETORES DA PREFEITURA MUNICIPAL DE SÃO JOÃO DAS DUAS PONTES, CONFORME ESPECIFICAÇÕES E CONDIÇÕES ESTABELECIDAS NO TERMO DE REFERÊNCIA.</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>1217853.48</v>
+        <v>1344360.65</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-08-26T08:00:00</t>
+          <t>2026-09-02T08:00:00</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-10T08:30:00</t>
+          <t>2026-09-15T08:59:00</t>
         </is>
       </c>
       <c r="K18" t="n">
@@ -36463,19 +36463,19 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE SANTA ALBERTINA</t>
+          <t>MUNICIPIO DE SAO JOAO DAS DUAS PONTES</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>51842177000176-1-000009/2026</t>
+          <t>65712002000159-1-000025/2026</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Populina</t>
+          <t>Aspásia</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -36483,7 +36483,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -36496,20 +36496,20 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Registro de preços para futura e eventual aquisição, com instalação, de playgrounds, brinquedos infantis, equipamentos recreativos e mobiliário de apoio, destinados a praças, parques, escolas e demais espaços públicos municipais de Populina/SP.</t>
+          <t>Registro de preços para eventual contratação de empresa para a locação de brinquedos infláveis, disponibilização do Carretão da Alegria e prestação de serviços de carrinho de pipoca, algodão-doce e churros, incluindo transporte, montagem, instalação, operação e acompanhamento, para realização dos eventos promovidos pelo município de Aspásia-SP.</t>
         </is>
       </c>
       <c r="H19" t="n">
-        <v>2237327.4</v>
+        <v>122371.45</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-08-26T08:00:00</t>
+          <t>2026-08-28T08:00:00</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-11T08:25:00</t>
+          <t>2026-09-16T08:00:00</t>
         </is>
       </c>
       <c r="K19" t="n">
@@ -36517,24 +36517,24 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>https://bllcompras.com/Process/ProcessView?param1=[gkz]bLezG7PRY7kJ7HUtk7XrKi8hDh5fHQ8eun9/MHtyLQ04gxN3BLr9J8rvwQ/KeKtJFkMnFHKfUVMoJVWokccurrPTtpguXan7eH8UyRlHbHw=</t>
+          <t>https://bllcompras.com/Process/ProcessView?param1=[gkz]ybDTuhueE/wN6RpDwRmykLkLev79jz7z/zawjhjmDhcthLfaFu7pRiWqaR6SCOuQZDVfdixJxj1eWqMt2SwDQrc1q75ShfBleAkQ/X3sWMg=</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE POPULINA</t>
+          <t>MUNICIPIO DE ASPASIA</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>01611210000189-1-000039/2026</t>
+          <t>46611117000102-1-000034/2026</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Vitória Brasil</t>
+          <t>Urânia</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -36542,12 +36542,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>019</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Pregão - Eletrônico</t>
+          <t>Credenciamento</t>
         </is>
       </c>
       <c r="F20" t="n">
@@ -36555,53 +36555,48 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Contratação de empresa especializada para prestação continuada de serviços técnicos profissionais de engenharia civil, mediante disponibilização de profissional legalmente habilitado e registrado no CREA, para atendimento das demandas técnicas do Município de Vitória Brasil/SP, conforme especificações e condições estabelecidas no Termo de Referência.</t>
+          <t>CONTRATAÇÃO PARA AGRICULTURA FAMILIAR</t>
         </is>
       </c>
       <c r="H20" t="n">
-        <v>72000</v>
+        <v>785709.02</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-08-26T07:00:00</t>
+          <t>2026-08-27T09:00:00</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-11T07:00:00</t>
+          <t>2026-09-16T09:00:00</t>
         </is>
       </c>
       <c r="K20" t="n">
         <v>0</v>
       </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>https://bllcompras.com/Process/ProcessView?param1=[gkz]vQQuhlx2Pl8lkR4jblHBp53gsyiYaUO5R79qyHqzmfBAXAgoaWDIYQNetaVTV6wokPn_VoeOaP31PgAi8W9JkZoK42fYxR_Q3rLDM3pZlz4=</t>
-        </is>
-      </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE VITORIA BRASIL</t>
+          <t>MUNICIPIO DE URANIA</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>45138070000149-1-000794/2026</t>
+          <t>01611211000123-1-000050/2026</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Santa Fé do Sul</t>
+          <t>Santa Salete</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>22</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -36614,53 +36609,48 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Aquisição de material permanente do tipo arma de fogo, destinados ao aparelhamento da Guarda Civil Municipal</t>
+          <t>CONTRATAÇÃO DE EMPRESA PARA AQUISIÇÃO DOS ITENS FRACASSADOS DO PREGÃO ELETRÔNICO Nº 016/2026, REFERENTES AO FORNECIMENTO DE DIVERSOS MATERIAIS ESCOLARES, CONFORME ESPECIFICAÇÕES CONSTANTES NO TERMO DE REFERÊNCIA, DESTINADOS AO ATENDIMENTO DAS NECESSIDADES DO DEPARTAMENTO MUNICIPAL DE EDUCAÇÃO DO MUNICÍPIO DE SANTA SALETE/SP</t>
         </is>
       </c>
       <c r="H21" t="n">
-        <v>214982.55</v>
+        <v>80562.47</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-09-01T08:00:00</t>
+          <t>2026-09-02T08:30:00</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-14T08:00:00</t>
+          <t>2026-09-16T08:30:00</t>
         </is>
       </c>
       <c r="K21" t="n">
         <v>0</v>
       </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/compras/acompanhamento-compra?compra=98703305000012026</t>
-        </is>
-      </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE SANTA FE DO SUL</t>
+          <t>MUNICIPIO DE SANTA SALETE</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>46609731000130-1-000010/2026</t>
+          <t>01613202000171-1-000002/2026</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Palmeira d'Oeste</t>
+          <t>Nova Castilho</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0012/26</t>
+          <t>010</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -36673,20 +36663,20 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Registro de preço para futura e eventual aquisição e fornecimento de materiais hospitalares e injetáveis (ampolas) que serão utilizados nas Unidades Básicas de Saúde do município de Palmeira D’Oeste</t>
+          <t>Aquisição de Equipamentos</t>
         </is>
       </c>
       <c r="H22" t="n">
-        <v>1389925.25</v>
+        <v>135576.2</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-08-28T08:00:00</t>
+          <t>2026-09-03T08:30:00</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-15T07:55:00</t>
+          <t>2026-09-16T08:30:00</t>
         </is>
       </c>
       <c r="K22" t="n">
@@ -36694,19 +36684,19 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>https://bllcompras.com/Process/ProcessView?param1=[gkz]l2ky7JpCrcgDbj_wLQNaUs/Mz/47PiTcEIcmcwf6lBs4uuoJI5JXsJ_Ups37yV8xnqw04gNabtq9EQoZRGeClFx0zNFKTnizlwfbEv/M2IM=</t>
+          <t>https://bllcompras.com/Process/ProcessView?param1=[gkz]pBpu1ToEXvqoatStX5iXKa1wR44yORZ45qMl76FhGtut7rYep2kFZAJsG7zT4s6KjfRuhBqECni4Ntp8BZTF3SR2yHcdE1XmKhYrF0q8fXs=</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE PALMEIRA D'OESTE</t>
+          <t>MUNICIPIO DE NOVA CASTILHO</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>46611117000102-1-000035/2026</t>
+          <t>46611117000102-1-000036/2026</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -36719,7 +36709,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>024</t>
+          <t>023</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -36732,20 +36722,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Contratação de empresa especializada para prestações de serviços mecânicos com fornecimento de peças para os seguintes veículos da frota municipal: FORD CAMINHÃO PIPA– Placa BFY2619 e ONIBUS VOLARE DW9 – Placa FQL1B98, pertencentes ao Município de Urânia/SP.</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA A PRESTAÇÃO DE SERVIÇOS DE UM PROFESSOR DE EDUCAÇÃO FÍSICA PARA DESENVOLVER OFICINA DE TREINAMENTO DE FUTEBOL, PARA ATENDER ÀS NECESSIDADES DA SECRETARIA MUNICIPAL DE ESPORTE, CULTURA E TURISMO, CONFORME ESPECIFICAÇÕES E CONDIÇÕES CONSTANTES NO TERMO DE REFERÊNCIA (TR).</t>
         </is>
       </c>
       <c r="H23" t="n">
-        <v>35351.29</v>
+        <v>54102</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-09-01T09:00:00</t>
+          <t>2026-09-02T09:00:00</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-15T08:50:00</t>
+          <t>2026-09-18T08:50:00</t>
         </is>
       </c>
       <c r="K23" t="n">
@@ -36753,7 +36743,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>https://bllcompras.com/Process/ProcessView?param1=[gkz]jqtYlnxx02/zyCYX3kMbJ7UZt703DK0ewrudwGqCXRJlwWEUMxkpBqjwyPOSwmbnA_gUzilGP86b0FjDqmllHvDzbYRj6mOcMGzhbs8wzJM=</t>
+          <t>https://bllcompras.com/Process/ProcessView?param1=[gkz]MqJvUmc8o9dSkJykigz/1cyMrTRnSna109cJUoZkSEcOTAiANY2Xa_CPsRe70qWaL23tnYxoNIrYc0YjaRsvXGZ3AoqEQbTwNpnZ1xe1vrc=</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -36765,12 +36755,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>45116712000109-1-000050/2026</t>
+          <t>45115391000128-1-000015/2026</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>São João das Duas Pontes</t>
+          <t>Guarani d'Oeste</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -36778,7 +36768,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>004</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -36791,40 +36781,45 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>ELABORAÇÃO DE ATA DE REGISTRO DE PREÇOS PARA FUTURA E EVENTUAL AQUISIÇÃO PARCELADA DE MEDICAMENTOS, DESTINADOS AO ABASTECIMENTO DA FARMÁCIA MUNICIPAL E AO ATENDI-MENTO DOS PACIENTES USUÁRIOS DO SUS DO MUNICÍPIO DE SÃO JOÃO DAS DUAS PONTES/SP, PELO PERÍODO ESTIMADO DE 12 (DOZE) MESES’’.</t>
+          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA SERVIÇOS DE DISPOSIÇÃO FINAL DOS RESÍDUOS SÓLIDOS DO MUNICÍPIO DE GUARANI D’OESTE/SP.</t>
         </is>
       </c>
       <c r="H24" t="n">
-        <v>118801</v>
+        <v>117000</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-09-02T08:00:00</t>
+          <t>2026-09-01T08:00:00</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-15T08:59:00</t>
+          <t>2026-09-18T08:30:00</t>
         </is>
       </c>
       <c r="K24" t="n">
         <v>0</v>
       </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>https://bllcompras.com/Process/ProcessView?param1=[gkz]jInmuOgu0_YB_dquijP_RZGWfyVr/eOdywIFnHRtIlyp5ms9JHxexy6A9a/qz4Pb/k9roi/SWuR_tSiwC0zGrkZi8qFpcI9cr/A2VKEm8Bs=</t>
+        </is>
+      </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE SAO JOAO DAS DUAS PONTES</t>
+          <t>MUNICIPIO DE GUARANI D'OESTE</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>45116712000109-1-000051/2026</t>
+          <t>47842836000105-1-000158/2026</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>São João das Duas Pontes</t>
+          <t>Fernandópolis</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -36832,7 +36827,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>43</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -36845,11 +36840,11 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>ELABORAÇÃO DE ATA DE REGISTRO DE PREÇOS PARA FUTURA E EVENTUAL AQUISIÇÃO DE EQUIPAMENTOS E DISPOSITIVOS TECNOLÓGICOS, INCLUINDO ITENS FRACASSADOS E NOVOS, PARA ATENDIMENTO DAS NECESSIDADES DOS DIVERSOS SETORES DA PREFEITURA MUNICIPAL DE SÃO JOÃO DAS DUAS PONTES, CONFORME ESPECIFICAÇÕES E CONDIÇÕES ESTABELECIDAS NO TERMO DE REFERÊNCIA.</t>
+          <t>ELABORAÇÃO DE ATA DE REGISTRO DE PREÇOS PARA AQUISIÇÃO DE GARRAFAS TÉRMICAS DE 1 LITRO E BATERIAS NÃO RECARREGÁVEIS DESTINADAS AOS AGENTES COMUNITÁRIOS DE SAÚDE E AGENTES DE COMBATE ÀS ENDEMIAS DA SECRETARIA MUNICIPAL DE SAÚDE DE FERNANDÓPOLIS/SP, COM PREVISÃO DE CONSUMO NO DECORRER DE 12 (DOZE) MESES</t>
         </is>
       </c>
       <c r="H25" t="n">
-        <v>1344360.65</v>
+        <v>24897.5</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -36858,27 +36853,32 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-15T08:59:00</t>
+          <t>2026-09-18T08:29:00</t>
         </is>
       </c>
       <c r="K25" t="n">
         <v>0</v>
       </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/compras/acompanhamento-compra?compra=98641105000432026</t>
+        </is>
+      </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE SAO JOAO DAS DUAS PONTES</t>
+          <t>MUNICIPIO DE FERNANDOPOLIS</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>65712002000159-1-000025/2026</t>
+          <t>01611211000123-1-000049/2026</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Aspásia</t>
+          <t>Santa Salete</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -36886,7 +36886,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>25</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -36899,58 +36899,53 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Registro de preços para eventual contratação de empresa para a locação de brinquedos infláveis, disponibilização do Carretão da Alegria e prestação de serviços de carrinho de pipoca, algodão-doce e churros, incluindo transporte, montagem, instalação, operação e acompanhamento, para realização dos eventos promovidos pelo município de Aspásia-SP.</t>
+          <t>Contratação de empresa especializada para prestação de serviços de Fonoaudiologia e Terapia Ocupacional, compreendendo 20 (vinte) horas mensais de atendimento para cada profissional, destinados ao atendimento de paciente do Município de Santa Salete/SP, em cumprimento à decisão judicial proferida nos autos do Agravo de Instrumento nº 2176644-50.2026.8.26.0000, conforme indicação da equipe multiprofissional responsável pelo acompanhamento da paciente.</t>
         </is>
       </c>
       <c r="H26" t="n">
-        <v>122371.45</v>
+        <v>79585.8</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-08-28T08:00:00</t>
+          <t>2026-09-02T08:30:00</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-16T08:00:00</t>
+          <t>2026-09-18T08:30:00</t>
         </is>
       </c>
       <c r="K26" t="n">
         <v>0</v>
       </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>https://bllcompras.com/Process/ProcessView?param1=[gkz]ybDTuhueE/wN6RpDwRmykLkLev79jz7z/zawjhjmDhcthLfaFu7pRiWqaR6SCOuQZDVfdixJxj1eWqMt2SwDQrc1q75ShfBleAkQ/X3sWMg=</t>
-        </is>
-      </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE ASPASIA</t>
+          <t>MUNICIPIO DE SANTA SALETE</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>46611117000102-1-000034/2026</t>
+          <t>45138070000149-1-000806/2026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Urânia</t>
+          <t>Santa Fé do Sul</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>102</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Credenciamento</t>
+          <t>Pregão - Eletrônico</t>
         </is>
       </c>
       <c r="F27" t="n">
@@ -36958,48 +36953,53 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO PARA AGRICULTURA FAMILIAR</t>
+          <t>Contratação de empresa especializada em manejo arbóreo dentro do limite territorial de Santa Fé do Sul</t>
         </is>
       </c>
       <c r="H27" t="n">
-        <v>785709.02</v>
+        <v>3304600</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-08-27T09:00:00</t>
+          <t>2026-09-03T08:00:00</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-09-16T09:00:00</t>
+          <t>2026-09-18T08:00:00</t>
         </is>
       </c>
       <c r="K27" t="n">
         <v>0</v>
       </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/compras/acompanhamento-compra?compra=98703305001022026</t>
+        </is>
+      </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE URANIA</t>
+          <t>MUNICIPIO DE SANTA FE DO SUL</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>01611211000123-1-000050/2026</t>
+          <t>45138070000149-1-000808/2026</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Santa Salete</t>
+          <t>Santa Fé do Sul</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>44</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -37012,48 +37012,53 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA PARA AQUISIÇÃO DOS ITENS FRACASSADOS DO PREGÃO ELETRÔNICO Nº 016/2026, REFERENTES AO FORNECIMENTO DE DIVERSOS MATERIAIS ESCOLARES, CONFORME ESPECIFICAÇÕES CONSTANTES NO TERMO DE REFERÊNCIA, DESTINADOS AO ATENDIMENTO DAS NECESSIDADES DO DEPARTAMENTO MUNICIPAL DE EDUCAÇÃO DO MUNICÍPIO DE SANTA SALETE/SP</t>
+          <t>Registro de Preços para a eventual e futura contratação de empresa especializada na prestação de Serviços de Acolhimento Institucional (Casa Lar) – Cuidador Social, de forma contínua e ininterrupta (24 horas diárias), pelo período de 12 (doze) meses, a fim de atender às demandas da Secretaria Municipal de Assistência Social do Município de Santa Fé do Sul/SP, conforme especificações, condições e quantitativos constantes no Edital e seus anexos.</t>
         </is>
       </c>
       <c r="H28" t="n">
-        <v>80562.47</v>
+        <v>1153692</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-09-02T08:30:00</t>
+          <t>2026-09-02T09:00:00</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-09-16T08:30:00</t>
+          <t>2026-09-18T09:00:00</t>
         </is>
       </c>
       <c r="K28" t="n">
         <v>0</v>
       </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>https://bllcompras.com/Process/ProcessView?param1=[gkz]/CmfpGhytjQ86nEur6pI0vxA1RabGATCTXzld4gfF6AbTpiSSmM4bMLVDnfjQ5cLn2dn4G4Brm43OZiEQl039/968_HFwLH4kw9VmdoGfTw=</t>
+        </is>
+      </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE SANTA SALETE</t>
+          <t>MUNICIPIO DE SANTA FE DO SUL</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>46611117000102-1-000036/2026</t>
+          <t>45138070000149-1-000807/2026</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Urânia</t>
+          <t>Santa Fé do Sul</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>023</t>
+          <t>42</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -37066,20 +37071,20 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA A PRESTAÇÃO DE SERVIÇOS DE UM PROFESSOR DE EDUCAÇÃO FÍSICA PARA DESENVOLVER OFICINA DE TREINAMENTO DE FUTEBOL, PARA ATENDER ÀS NECESSIDADES DA SECRETARIA MUNICIPAL DE ESPORTE, CULTURA E TURISMO, CONFORME ESPECIFICAÇÕES E CONDIÇÕES CONSTANTES NO TERMO DE REFERÊNCIA (TR).</t>
+          <t>REGISTRO DE PREÇOS para futura e eventual aquisição de materiais recreativos, jogos educativos e brinquedos, destinados ao atendimento das necessidades das Secretarias do Município de Santa Fé do Sul/SP, pelo período de 12 (doze) meses, com fornecimento de forma parcelada, conforme a demanda, observadas as condições, quantidades e exigências estabelecidas no Edital e em seus anexos.</t>
         </is>
       </c>
       <c r="H29" t="n">
-        <v>54102</v>
+        <v>498226.58</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-09-02T09:00:00</t>
+          <t>2026-09-03T08:00:00</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-09-18T08:50:00</t>
+          <t>2026-09-21T08:00:00</t>
         </is>
       </c>
       <c r="K29" t="n">
@@ -37087,24 +37092,24 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>https://bllcompras.com/Process/ProcessView?param1=[gkz]MqJvUmc8o9dSkJykigz/1cyMrTRnSna109cJUoZkSEcOTAiANY2Xa_CPsRe70qWaL23tnYxoNIrYc0YjaRsvXGZ3AoqEQbTwNpnZ1xe1vrc=</t>
+          <t>https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/compras/acompanhamento-compra?compra=98703305000422026</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE URANIA</t>
+          <t>MUNICIPIO DE SANTA FE DO SUL</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>45115391000128-1-000015/2026</t>
+          <t>47842836000105-1-000159/2026</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Guarani d'Oeste</t>
+          <t>Fernandópolis</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -37112,7 +37117,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>004</t>
+          <t>45</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -37125,20 +37130,20 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA SERVIÇOS DE DISPOSIÇÃO FINAL DOS RESÍDUOS SÓLIDOS DO MUNICÍPIO DE GUARANI D’OESTE/SP.</t>
+          <t>“ELABORAÇÃO DE ATA DE REGISTRO DE PREÇOS PARA AQUISIÇÃO DE RAÇÃO ANIMAL DESTINADA À EMEFA “MELVIN JONES”, COM PREVISÃO DE CONSUMO NO DECORRER DE 12 (DOZE) MESES”</t>
         </is>
       </c>
       <c r="H30" t="n">
-        <v>117000</v>
+        <v>77510.78</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-09-01T08:00:00</t>
+          <t>2026-09-04T08:00:00</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-18T08:30:00</t>
+          <t>2026-09-21T08:29:00</t>
         </is>
       </c>
       <c r="K30" t="n">
@@ -37146,24 +37151,24 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>https://bllcompras.com/Process/ProcessView?param1=[gkz]jInmuOgu0_YB_dquijP_RZGWfyVr/eOdywIFnHRtIlyp5ms9JHxexy6A9a/qz4Pb/k9roi/SWuR_tSiwC0zGrkZi8qFpcI9cr/A2VKEm8Bs=</t>
+          <t>https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/compras/acompanhamento-compra?compra=98641105000452026</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE GUARANI D'OESTE</t>
+          <t>MUNICIPIO DE FERNANDOPOLIS</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>47842836000105-1-000158/2026</t>
+          <t>01611211000123-1-000051/2026</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Fernandópolis</t>
+          <t>Santa Salete</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -37171,7 +37176,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>23</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -37184,45 +37189,40 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>ELABORAÇÃO DE ATA DE REGISTRO DE PREÇOS PARA AQUISIÇÃO DE GARRAFAS TÉRMICAS DE 1 LITRO E BATERIAS NÃO RECARREGÁVEIS DESTINADAS AOS AGENTES COMUNITÁRIOS DE SAÚDE E AGENTES DE COMBATE ÀS ENDEMIAS DA SECRETARIA MUNICIPAL DE SAÚDE DE FERNANDÓPOLIS/SP, COM PREVISÃO DE CONSUMO NO DECORRER DE 12 (DOZE) MESES</t>
+          <t>AQUISIÇÃO GÊNEROS ALIMENTÍCIOS, MATERIAIS DE LIMPEZA, EMBALAGENS E PRODUTOS DE HIGIENE, PARA ATENDER A DEMANDA DOS DIVERSOS SETORES DA MUNICIPALIDADE, COM FORNECIMENTO DE FORMA PARCELADA, DIÁRIA, CONFORME SOLICITAÇÃO, PELO PERÍODO DE 12 (DOZE) MESES, CONFORME TERMO DE REFERÊNCIA</t>
         </is>
       </c>
       <c r="H31" t="n">
-        <v>24897.5</v>
+        <v>1937025.05</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-09-02T08:00:00</t>
+          <t>2026-09-08T08:30:00</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-18T08:29:00</t>
+          <t>2026-09-21T08:30:00</t>
         </is>
       </c>
       <c r="K31" t="n">
         <v>0</v>
       </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/compras/acompanhamento-compra?compra=98641105000432026</t>
-        </is>
-      </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE FERNANDOPOLIS</t>
+          <t>MUNICIPIO DE SANTA SALETE</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>01611211000123-1-000049/2026</t>
+          <t>47842836000105-1-000160/2026</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Santa Salete</t>
+          <t>Fernandópolis</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -37230,7 +37230,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>44</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -37243,48 +37243,53 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Contratação de empresa especializada para prestação de serviços de Fonoaudiologia e Terapia Ocupacional, compreendendo 20 (vinte) horas mensais de atendimento para cada profissional, destinados ao atendimento de paciente do Município de Santa Salete/SP, em cumprimento à decisão judicial proferida nos autos do Agravo de Instrumento nº 2176644-50.2026.8.26.0000, conforme indicação da equipe multiprofissional responsável pelo acompanhamento da paciente.</t>
+          <t>ELABORAÇÃO DE ATA DE REGISTRO DE PREÇOS PARA AQUISIÇÃO DE GÊNEROS ALIMENTÍCIOS, COM PREVISÃO DE CONSUMO NO DECORRER DE 12 (DOZE) MESES</t>
         </is>
       </c>
       <c r="H32" t="n">
-        <v>79585.8</v>
+        <v>646230.7</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-09-02T08:30:00</t>
+          <t>2026-09-04T08:00:00</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-09-18T08:30:00</t>
+          <t>2026-09-22T08:29:00</t>
         </is>
       </c>
       <c r="K32" t="n">
         <v>0</v>
       </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/compras/acompanhamento-compra?compra=98641105000442026</t>
+        </is>
+      </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE SANTA SALETE</t>
+          <t>MUNICIPIO DE FERNANDOPOLIS</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>45138070000149-1-000806/2026</t>
+          <t>47842836000105-1-000161/2026</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Santa Fé do Sul</t>
+          <t>Fernandópolis</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>102</t>
+          <t>46</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -37297,20 +37302,20 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Contratação de empresa especializada em manejo arbóreo dentro do limite territorial de Santa Fé do Sul</t>
+          <t>AQUISIÇÃO DE CESTO METÁLICO PARA DUAS PESSOAS ACOPLADO PARA GUINDASTE/MUNCK</t>
         </is>
       </c>
       <c r="H33" t="n">
-        <v>3304600</v>
+        <v>14730</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-09-03T08:00:00</t>
+          <t>2026-09-08T08:00:00</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-09-18T08:00:00</t>
+          <t>2026-09-23T08:29:00</t>
         </is>
       </c>
       <c r="K33" t="n">
@@ -37318,32 +37323,32 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/compras/acompanhamento-compra?compra=98703305001022026</t>
+          <t>https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/compras/acompanhamento-compra?compra=98641105000462026</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE SANTA FE DO SUL</t>
+          <t>MUNICIPIO DE FERNANDOPOLIS</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>45138070000149-1-000808/2026</t>
+          <t>47842836000105-1-000162/2026</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Santa Fé do Sul</t>
+          <t>Fernandópolis</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>47</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -37356,20 +37361,20 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Registro de Preços para a eventual e futura contratação de empresa especializada na prestação de Serviços de Acolhimento Institucional (Casa Lar) – Cuidador Social, de forma contínua e ininterrupta (24 horas diárias), pelo período de 12 (doze) meses, a fim de atender às demandas da Secretaria Municipal de Assistência Social do Município de Santa Fé do Sul/SP, conforme especificações, condições e quantitativos constantes no Edital e seus anexos.</t>
+          <t>ELABORAÇÃO DE ATA DE REGISTRO DE PREÇOS PARA CONTRATAÇÃO DE EMPRESA ESPECIALIZADA NA PRESTAÇÃO DE SERVIÇOS DE DIAGNÓSTICO POR IMAGEM ODONTOLÓGICA, COMPREENDENDO A REALIZAÇÃO DE TOMOGRAFIA COMPUTADORIZADA DE FEIXE CÔNICO (CONE BEAM) DE MAXILA E DE MANDÍBULA, RADIOGRAFIA PANORÂMICA E RADIOGRAFIA PERIAPICAL, DESTINADOS AO ATENDIMENTO DOS PACIENTES ENCAMINHADOS PELA REDE MUNICIPAL DE SAÚDE DE FERNANDÓPOLIS/SP, COM PREVISÃO DE CONSUMO NO DECORRER DE 12 (DOZE) MESES</t>
         </is>
       </c>
       <c r="H34" t="n">
-        <v>1153692</v>
+        <v>547616.76</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-09-02T09:00:00</t>
+          <t>2026-09-08T08:00:00</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-09-18T09:00:00</t>
+          <t>2026-09-25T08:29:00</t>
         </is>
       </c>
       <c r="K34" t="n">
@@ -37377,32 +37382,32 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>https://bllcompras.com/Process/ProcessView?param1=[gkz]/CmfpGhytjQ86nEur6pI0vxA1RabGATCTXzld4gfF6AbTpiSSmM4bMLVDnfjQ5cLn2dn4G4Brm43OZiEQl039/968_HFwLH4kw9VmdoGfTw=</t>
+          <t>https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/compras/acompanhamento-compra?compra=98641105000472026</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE SANTA FE DO SUL</t>
+          <t>MUNICIPIO DE FERNANDOPOLIS</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>45138070000149-1-000807/2026</t>
+          <t>46377800000127-1-003500/2026</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Santa Fé do Sul</t>
+          <t>Fernandópolis</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>47</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -37415,20 +37420,20 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>REGISTRO DE PREÇOS para futura e eventual aquisição de materiais recreativos, jogos educativos e brinquedos, destinados ao atendimento das necessidades das Secretarias do Município de Santa Fé do Sul/SP, pelo período de 12 (doze) meses, com fornecimento de forma parcelada, conforme a demanda, observadas as condições, quantidades e exigências estabelecidas no Edital e em seus anexos.</t>
+          <t>Prestação de serviço de manutenção preventiva e corretiva de viaturas</t>
         </is>
       </c>
       <c r="H35" t="n">
-        <v>498226.58</v>
+        <v>54097</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-09-03T08:00:00</t>
+          <t>2026-09-02T08:00:00</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-09-21T08:00:00</t>
+          <t>2026-09-28T09:00:00</t>
         </is>
       </c>
       <c r="K35" t="n">
@@ -37436,37 +37441,37 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/compras/acompanhamento-compra?compra=98703305000422026</t>
+          <t>https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/compras/acompanhamento-compra?compra=18014705000472026</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE SANTA FE DO SUL</t>
+          <t>SAO PAULO SECRETARIA DA SEGURANCA PUBLICA</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>46377800000127-1-003500/2026</t>
+          <t>45131885000104-1-000139/2025</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Fernandópolis</t>
+          <t>Jales</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>02</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Pregão - Eletrônico</t>
+          <t>Credenciamento</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -37474,20 +37479,20 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Prestação de serviço de manutenção preventiva e corretiva de viaturas</t>
+          <t>Visa- se o Chamamento Público que tem por objeto o credenciamento de pessoas jurídicas para a prestação de serviços de Fonoaudiólogo, Tradutor e Interpretes de Libras e Médicos: Clínico Geral, Ginecologista, Pediatra, Infectologista, Auditor/Regulador, Diretor Técnico e Psiquiatra, com entrega parcelada, por tempo determinado, conforme Termo de Referência – Anexo I.</t>
         </is>
       </c>
       <c r="H36" t="n">
-        <v>54097</v>
+        <v>5354131.2</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2026-09-02T08:00:00</t>
+          <t>2025-10-15T08:00:00</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-09-28T09:00:00</t>
+          <t>2026-10-14T08:00:00</t>
         </is>
       </c>
       <c r="K36" t="n">
@@ -37495,32 +37500,32 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/compras/acompanhamento-compra?compra=18014705000472026</t>
+          <t>https://bllcompras.com/Process/ProcessView?param1=[gkz]lvbKyYvKIZiklLxiAv8yLXpH61nfdQ27zWjL4LgDP9TI_EL2tTI7HuwRFC9TLbbPEkTpieh_v08t375hW7Ho0/56cHYOdyQiOLOgx/mkV0g=</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>SAO PAULO SECRETARIA DA SEGURANCA PUBLICA</t>
+          <t>MUNICIPIO DE JALES</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>45131885000104-1-000139/2025</t>
+          <t>47842836000105-1-000131/2025</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Jales</t>
+          <t>Fernandópolis</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>197</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -37532,65 +37537,6 @@
         <v>0</v>
       </c>
       <c r="G37" t="inlineStr">
-        <is>
-          <t>Visa- se o Chamamento Público que tem por objeto o credenciamento de pessoas jurídicas para a prestação de serviços de Fonoaudiólogo, Tradutor e Interpretes de Libras e Médicos: Clínico Geral, Ginecologista, Pediatra, Infectologista, Auditor/Regulador, Diretor Técnico e Psiquiatra, com entrega parcelada, por tempo determinado, conforme Termo de Referência – Anexo I.</t>
-        </is>
-      </c>
-      <c r="H37" t="n">
-        <v>5354131.2</v>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>2025-10-15T08:00:00</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>2026-10-14T08:00:00</t>
-        </is>
-      </c>
-      <c r="K37" t="n">
-        <v>0</v>
-      </c>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>https://bllcompras.com/Process/ProcessView?param1=[gkz]lvbKyYvKIZiklLxiAv8yLXpH61nfdQ27zWjL4LgDP9TI_EL2tTI7HuwRFC9TLbbPEkTpieh_v08t375hW7Ho0/56cHYOdyQiOLOgx/mkV0g=</t>
-        </is>
-      </c>
-      <c r="M37" t="inlineStr">
-        <is>
-          <t>MUNICIPIO DE JALES</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>47842836000105-1-000131/2025</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Fernandópolis</t>
-        </is>
-      </c>
-      <c r="C38" t="n">
-        <v>0</v>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>197</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Credenciamento</t>
-        </is>
-      </c>
-      <c r="F38" t="n">
-        <v>0</v>
-      </c>
-      <c r="G38" t="inlineStr">
         <is>
           <t>CONTRATAÇÃO DE EMPRESA ESPECIALIZADA, POR MEIO DE CREDENCIAMENTO, PARA PRESTAÇÃO DE SERVIÇOS DE ASSISTÊNCIA À SAÚDE SUPLEMENTAR NA MODALIDADE DE PLANO DE SAÚDE COLETIVO EMPRESARIAL OU COLETIVO
 POR ADESÃO, COM SEGMENTAÇÃO AMBULATORIAL E HOSPITALAR COM OBSTETRÍCIA, PARA OS
@@ -37599,17 +37545,71 @@
 SERVIÇO E A LIBERDADE DE ESCOLHA DOS BENEFICIÁRIOS</t>
         </is>
       </c>
+      <c r="H37" t="n">
+        <v>2436910.8</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>2025-10-15T08:30:00</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>2026-10-14T17:00:00</t>
+        </is>
+      </c>
+      <c r="K37" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>MUNICIPIO DE FERNANDOPOLIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>45131885000104-1-000450/2026</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Jales</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Concorrência - Presencial</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Contratação de serviços de publicidade prestados por intermédio de agência de propaganda, abrangendo o conjunto de atividades realizadas de forma integrada, para atendimento às necessidades de comunicação da Prefeitura Municipal de Jales - SP, por tempo determinado, conforme condições estabelecidas no Termo de Referência – Anexo I e Briefing – Anexo II.</t>
+        </is>
+      </c>
       <c r="H38" t="n">
-        <v>2436910.8</v>
+        <v>780000</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2025-10-15T08:30:00</t>
+          <t>2026-09-04T08:30:00</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-10-14T17:00:00</t>
+          <t>2026-10-29T09:30:00</t>
         </is>
       </c>
       <c r="K38" t="n">
@@ -37617,7 +37617,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>MUNICIPIO DE FERNANDOPOLIS</t>
+          <t>MUNICIPIO DE JALES</t>
         </is>
       </c>
     </row>
@@ -37785,7 +37785,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -37845,7 +37845,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -37905,7 +37905,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -37965,7 +37965,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -38025,7 +38025,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -38085,7 +38085,7 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -38145,7 +38145,7 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -38205,7 +38205,7 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -38265,7 +38265,7 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -38325,7 +38325,7 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -38385,7 +38385,7 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -38445,7 +38445,7 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -38505,7 +38505,7 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -38565,7 +38565,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -38625,7 +38625,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -38685,7 +38685,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -38745,7 +38745,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -38805,7 +38805,7 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -38865,7 +38865,7 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -38925,7 +38925,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -38985,7 +38985,7 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -39045,7 +39045,7 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
@@ -39105,7 +39105,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -39165,7 +39165,7 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -39225,7 +39225,7 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
@@ -39285,7 +39285,7 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
@@ -39345,7 +39345,7 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -39405,7 +39405,7 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
@@ -39465,7 +39465,7 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -39525,7 +39525,7 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
@@ -39585,7 +39585,7 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
@@ -39645,7 +39645,7 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
@@ -39705,7 +39705,7 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -39765,7 +39765,7 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
@@ -39825,7 +39825,7 @@
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
@@ -39885,7 +39885,7 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -39945,7 +39945,7 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
@@ -40005,7 +40005,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -40065,7 +40065,7 @@
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
@@ -40125,7 +40125,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -40185,7 +40185,7 @@
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
@@ -40245,7 +40245,7 @@
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R43" t="inlineStr">
@@ -40305,7 +40305,7 @@
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R44" t="inlineStr">
@@ -40365,7 +40365,7 @@
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R45" t="inlineStr">
@@ -40425,7 +40425,7 @@
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
@@ -40485,7 +40485,7 @@
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R47" t="inlineStr">
@@ -40545,7 +40545,7 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
@@ -40605,7 +40605,7 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
@@ -40665,7 +40665,7 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
@@ -40725,7 +40725,7 @@
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
@@ -40785,7 +40785,7 @@
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
@@ -40845,7 +40845,7 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
@@ -40905,7 +40905,7 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
@@ -40965,7 +40965,7 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
@@ -41025,7 +41025,7 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R56" t="inlineStr">
@@ -41085,7 +41085,7 @@
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="R57" t="inlineStr">
@@ -42736,7 +42736,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -42778,102 +42778,1428 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>3</v>
+        <v>40</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>proposta 3532868 mod=6</t>
+          <t>itens 01611210000189/2026/39</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/api/consulta/v1/contratacoes/proposta</t>
-        </is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/01611210000189/compras/2026/39/itens</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>503</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>ReadTimeout: HTTPSConnectionPool(host='pncp.gov.br', port=443): Read timed out. (read timeout=45)</t>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-09-03T09:26:08+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-02T09:41:05+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>proposta 3547205 mod=7</t>
+          <t>itens 46611117000102/2026/34</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://pncp.gov.br/api/consulta/v1/contratacoes/proposta?dataFinal=20261101&amp;codigoModalidadeContratacao=7&amp;codigoMunicipioIbge=3547205&amp;tamanhoPagina=50&amp;pagina=1</t>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/46611117000102/compras/2026/34/itens</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>HTTP 500: Erro na comunicação com o banco de dados.</t>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-09-02T09:41:05+00:00</t>
+          <t>2026-09-07T09:37:26+00:00</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1</v>
+        <v>38</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>itens 46611117000102/2026/36</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/46611117000102/compras/2026/36/itens</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>503</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>37</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>itens 46611117000102/2026/35</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/46611117000102/compras/2026/35/itens</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>502</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 502: &lt;html&gt;&lt;body&gt;&lt;h1&gt;502 Bad Gateway&lt;/h1&gt;
+The server returned an invalid or incomplete response.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>36</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>itens 45139482000101/2026/13</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/45139482000101/compras/2026/13/itens</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>503</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>35</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>itens 45116712000109/2026/51</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/45116712000109/compras/2026/51/itens</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>503</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>34</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>itens 45116712000109/2026/50</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/45116712000109/compras/2026/50/itens</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>503</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>33</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>itens 45138088000140/2026/5</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/45138088000140/compras/2026/5/itens</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>503</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>32</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>itens 01611211000123/2026/51</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/01611211000123/compras/2026/51/itens</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>503</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>31</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>itens 01611211000123/2026/50</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/01611211000123/compras/2026/50/itens</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>503</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>30</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>itens 01611211000123/2026/49</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/01611211000123/compras/2026/49/itens</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>503</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>29</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>itens 45135530000185/2026/43</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/45135530000185/compras/2026/43/itens</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>503</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>28</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>itens 45135043000112/2026/44</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/45135043000112/compras/2026/44/itens</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>503</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>27</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>itens 51842177000176/2026/9</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/51842177000176/compras/2026/9/itens</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>503</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>26</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>itens 46609731000130/2026/10</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/46609731000130/compras/2026/10/itens</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>503</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>25</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>itens 46609731000130/2026/9</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/46609731000130/compras/2026/9/itens</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>503</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>24</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>itens 45116290000171/2026/71</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/45116290000171/compras/2026/71/itens</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>503</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>23</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>itens 45115391000128/2026/15</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/45115391000128/compras/2026/15/itens</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>503</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>22</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>itens 47842836000105/2025/131</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/47842836000105/compras/2025/131/itens</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>ConnectionError: ('Connection aborted.', RemoteDisconnected('Remote end closed connection without response'))</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>21</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>itens 47842836000105/2026/162</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/47842836000105/compras/2026/162/itens</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>503</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>itens 47842836000105/2026/161</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/47842836000105/compras/2026/161/itens</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>503</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>itens 47842836000105/2026/160</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/47842836000105/compras/2026/160/itens</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>503</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>18</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>itens 47842836000105/2026/159</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/47842836000105/compras/2026/159/itens</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>502</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 502: &lt;html&gt;&lt;body&gt;&lt;h1&gt;502 Bad Gateway&lt;/h1&gt;
+The server returned an invalid or incomplete response.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>17</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>itens 47842836000105/2026/158</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/47842836000105/compras/2026/158/itens</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>503</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>16</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>itens 46377800000127/2026/3566</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/46377800000127/compras/2026/3566/itens</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>503</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>15</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>itens 46377800000127/2026/3500</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/46377800000127/compras/2026/3500/itens</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>503</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>14</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>itens 47842836000105/2026/155</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/47842836000105/compras/2026/155/itens</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>503</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>13</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>itens 65712002000159/2026/27</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/65712002000159/compras/2026/27/itens</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>503</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>12</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>itens 65712002000159/2026/25</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/65712002000159/compras/2026/25/itens</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>503</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>11</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>itens 65712002000159/2026/23</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/65712002000159/compras/2026/23/itens</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>503</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>10</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>itens 45138070000149/2026/808</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/45138070000149/compras/2026/808/itens</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>502</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 502: &lt;html&gt;&lt;body&gt;&lt;h1&gt;502 Bad Gateway&lt;/h1&gt;
+The server returned an invalid or incomplete response.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>9</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>itens 45138070000149/2026/807</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/45138070000149/compras/2026/807/itens</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>503</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>8</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>itens 45138070000149/2026/806</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/45138070000149/compras/2026/806/itens</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>503</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>7</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>itens 45138070000149/2026/794</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/45138070000149/compras/2026/794/itens</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>503</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>6</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>itens 01613202000171/2026/2</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/01613202000171/compras/2026/2/itens</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>503</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>5</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>itens 45131885000104/2025/139</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/45131885000104/compras/2025/139/itens</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>503</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>4</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>itens 45131885000104/2026/450</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/pncp/v1/orgaos/45131885000104/compras/2026/450/itens</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>503</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTTP 503: &lt;html&gt;&lt;body&gt;&lt;h1&gt;503 Service Unavailable&lt;/h1&gt;
+No server is available to handle this request.
+&lt;/body&gt;&lt;/html&gt;
+</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2026-09-07T09:37:26+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>3</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-09-03T09:26:08+00:00</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>proposta 3532868 mod=6</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/consulta/v1/contratacoes/proposta</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>ReadTimeout: HTTPSConnectionPool(host='pncp.gov.br', port=443): Read timed out. (read timeout=45)</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2026-09-03T09:26:08+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>2</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
           <t>2026-09-02T09:41:05+00:00</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>proposta 3547205 mod=7</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://pncp.gov.br/api/consulta/v1/contratacoes/proposta?dataFinal=20261101&amp;codigoModalidadeContratacao=7&amp;codigoMunicipioIbge=3547205&amp;tamanhoPagina=50&amp;pagina=1</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>500</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>HTTP 500: Erro na comunicação com o banco de dados.</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2026-09-02T09:41:05+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>1</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-09-02T09:41:05+00:00</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
         <is>
           <t>proposta 3547403 mod=9</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>https://pncp.gov.br/api/consulta/v1/contratacoes/proposta?dataFinal=20261101&amp;codigoModalidadeContratacao=9&amp;codigoMunicipioIbge=3547403&amp;tamanhoPagina=50&amp;pagina=1</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="E41" t="n">
         <v>500</v>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F41" t="inlineStr">
         <is>
           <t>HTTP 500: Erro na comunicação com o banco de dados.</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G41" t="inlineStr">
         <is>
           <t>2026-09-02T09:41:05+00:00</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G4"/>
+  <autoFilter ref="A1:G41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>